<commit_message>
Lignin for wood and fine roots
</commit_message>
<xml_diff>
--- a/data-raw/SpParamsDefinition.xlsx
+++ b/data-raw/SpParamsDefinition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="367">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="747" uniqueCount="371">
   <si>
     <t xml:space="preserve">ParameterName</t>
   </si>
@@ -541,10 +541,22 @@
     <t xml:space="preserve">kJ/kg</t>
   </si>
   <si>
-    <t xml:space="preserve">LigninPercent</t>
+    <t xml:space="preserve">LeafLigninPercent</t>
   </si>
   <si>
     <t xml:space="preserve">Percent of lignin+cutin over dry weight in leaves</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WoodLigninPercent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percent of lignin+cutin over dry weight in wood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FineRootLigninPercent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Percent of lignin+cutin over dry weight in fine roots</t>
   </si>
   <si>
     <t xml:space="preserve">LeafAngle</t>
@@ -1886,7 +1898,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F1048576"/>
+  <dimension ref="A1:F157"/>
   <sheetFormatPr defaultColWidth="10.25" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.13"/>
@@ -3316,16 +3328,16 @@
         <v>175</v>
       </c>
       <c r="B76" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>176</v>
       </c>
-      <c r="C76" s="1" t="s">
-        <v>177</v>
-      </c>
       <c r="D76" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>178</v>
+        <v>150</v>
       </c>
       <c r="F76" s="1" t="n">
         <v>0</v>
@@ -3333,19 +3345,19 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>176</v>
+        <v>167</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="D77" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E77" s="5" t="s">
-        <v>178</v>
+        <v>150</v>
       </c>
       <c r="F77" s="1" t="n">
         <v>0</v>
@@ -3353,19 +3365,19 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>181</v>
       </c>
-      <c r="B78" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="C78" s="1" t="s">
+      <c r="D78" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E78" s="5" t="s">
         <v>182</v>
-      </c>
-      <c r="D78" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E78" s="5" t="s">
-        <v>70</v>
       </c>
       <c r="F78" s="1" t="n">
         <v>0</v>
@@ -3376,7 +3388,7 @@
         <v>183</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C79" s="1" t="s">
         <v>184</v>
@@ -3385,7 +3397,7 @@
         <v>43</v>
       </c>
       <c r="E79" s="5" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="F79" s="1" t="n">
         <v>0</v>
@@ -3393,19 +3405,19 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>186</v>
       </c>
-      <c r="B80" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="C80" s="1" t="s">
-        <v>187</v>
-      </c>
       <c r="D80" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>185</v>
+        <v>70</v>
       </c>
       <c r="F80" s="1" t="n">
         <v>0</v>
@@ -3413,19 +3425,19 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C81" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="B81" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="C81" s="1" t="s">
+      <c r="D81" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E81" s="5" t="s">
         <v>189</v>
-      </c>
-      <c r="D81" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E81" s="5" t="s">
-        <v>185</v>
       </c>
       <c r="F81" s="1" t="n">
         <v>0</v>
@@ -3436,7 +3448,7 @@
         <v>190</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="C82" s="1" t="s">
         <v>191</v>
@@ -3445,7 +3457,7 @@
         <v>43</v>
       </c>
       <c r="E82" s="5" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="F82" s="1" t="n">
         <v>0</v>
@@ -3453,46 +3465,50 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="B83" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C83" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="B83" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>195</v>
-      </c>
       <c r="D83" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E83" s="5"/>
+      <c r="E83" s="5" t="s">
+        <v>189</v>
+      </c>
       <c r="F83" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B84" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="D84" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E84" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="B84" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="D84" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E84" s="5"/>
       <c r="F84" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B85" s="6" t="s">
         <v>198</v>
-      </c>
-      <c r="B85" s="6" t="s">
-        <v>194</v>
       </c>
       <c r="C85" s="1" t="s">
         <v>199</v>
@@ -3500,22 +3516,20 @@
       <c r="D85" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E85" s="5" t="s">
-        <v>200</v>
-      </c>
+      <c r="E85" s="5"/>
       <c r="F85" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
+        <v>200</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C86" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="B86" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>202</v>
       </c>
       <c r="D86" s="1" t="s">
         <v>43</v>
@@ -3527,19 +3541,19 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B87" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C87" s="1" t="s">
         <v>203</v>
       </c>
-      <c r="B87" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C87" s="1" t="s">
+      <c r="D87" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E87" s="5" t="s">
         <v>204</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E87" s="5" t="s">
-        <v>205</v>
       </c>
       <c r="F87" s="1" t="n">
         <v>0</v>
@@ -3547,13 +3561,13 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C88" s="1" t="s">
         <v>206</v>
-      </c>
-      <c r="B88" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>207</v>
       </c>
       <c r="D88" s="1" t="s">
         <v>43</v>
@@ -3565,18 +3579,20 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="B89" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C89" s="1" t="s">
         <v>208</v>
       </c>
-      <c r="B89" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C89" s="1" t="s">
+      <c r="D89" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="D89" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E89" s="5"/>
       <c r="F89" s="1" t="n">
         <v>0</v>
       </c>
@@ -3586,7 +3602,7 @@
         <v>210</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>211</v>
@@ -3599,61 +3615,57 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
         <v>212</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C91" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="C91" s="1" t="s">
         <v>213</v>
       </c>
       <c r="D91" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E91" s="5" t="s">
-        <v>214</v>
-      </c>
+      <c r="E91" s="5"/>
       <c r="F91" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="B92" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C92" s="1" t="s">
         <v>215</v>
       </c>
-      <c r="B92" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C92" s="1" t="s">
+      <c r="D92" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E92" s="5"/>
+      <c r="F92" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="3" t="s">
         <v>216</v>
       </c>
-      <c r="D92" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E92" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="F92" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A93" s="3" t="s">
+      <c r="B93" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C93" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="B93" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C93" s="1" t="s">
+      <c r="D93" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E93" s="5" t="s">
         <v>218</v>
-      </c>
-      <c r="D93" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E93" s="5" t="s">
-        <v>219</v>
       </c>
       <c r="F93" s="1" t="n">
         <v>0</v>
@@ -3661,19 +3673,19 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="B94" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C94" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="B94" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C94" s="1" t="s">
-        <v>221</v>
-      </c>
       <c r="D94" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E94" s="5" t="s">
-        <v>100</v>
+        <v>218</v>
       </c>
       <c r="F94" s="1" t="n">
         <v>0</v>
@@ -3681,18 +3693,20 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="B95" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C95" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="B95" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C95" s="1" t="s">
+      <c r="D95" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E95" s="5" t="s">
         <v>223</v>
       </c>
-      <c r="D95" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E95" s="5"/>
       <c r="F95" s="1" t="n">
         <v>0</v>
       </c>
@@ -3702,7 +3716,7 @@
         <v>224</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C96" s="1" t="s">
         <v>225</v>
@@ -3711,7 +3725,7 @@
         <v>43</v>
       </c>
       <c r="E96" s="5" t="s">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="F96" s="1" t="n">
         <v>0</v>
@@ -3722,7 +3736,7 @@
         <v>226</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C97" s="1" t="s">
         <v>227</v>
@@ -3730,28 +3744,26 @@
       <c r="D97" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E97" s="5" t="s">
-        <v>228</v>
-      </c>
+      <c r="E97" s="5"/>
       <c r="F97" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C98" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="B98" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C98" s="1" t="s">
-        <v>230</v>
-      </c>
       <c r="D98" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E98" s="5" t="s">
-        <v>231</v>
+        <v>204</v>
       </c>
       <c r="F98" s="1" t="n">
         <v>0</v>
@@ -3759,19 +3771,19 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="B99" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="D99" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E99" s="5" t="s">
         <v>232</v>
-      </c>
-      <c r="B99" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C99" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="D99" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E99" s="5" t="s">
-        <v>200</v>
       </c>
       <c r="F99" s="1" t="n">
         <v>0</v>
@@ -3779,19 +3791,19 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="B100" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="B100" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C100" s="1" t="s">
+      <c r="D100" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E100" s="5" t="s">
         <v>235</v>
-      </c>
-      <c r="D100" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E100" s="5" t="s">
-        <v>200</v>
       </c>
       <c r="F100" s="1" t="n">
         <v>0</v>
@@ -3802,7 +3814,7 @@
         <v>236</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C101" s="1" t="s">
         <v>237</v>
@@ -3811,7 +3823,7 @@
         <v>43</v>
       </c>
       <c r="E101" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F101" s="1" t="n">
         <v>0</v>
@@ -3822,7 +3834,7 @@
         <v>238</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>239</v>
@@ -3831,7 +3843,7 @@
         <v>43</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="F102" s="1" t="n">
         <v>0</v>
@@ -3842,7 +3854,7 @@
         <v>240</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>241</v>
@@ -3851,7 +3863,7 @@
         <v>43</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>242</v>
+        <v>204</v>
       </c>
       <c r="F103" s="1" t="n">
         <v>0</v>
@@ -3859,19 +3871,19 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="B104" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C104" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="B104" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C104" s="1" t="s">
-        <v>244</v>
-      </c>
       <c r="D104" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>200</v>
+        <v>232</v>
       </c>
       <c r="F104" s="1" t="n">
         <v>0</v>
@@ -3879,19 +3891,19 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="B105" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C105" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="B105" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C105" s="1" t="s">
+      <c r="D105" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E105" s="5" t="s">
         <v>246</v>
-      </c>
-      <c r="D105" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E105" s="5" t="s">
-        <v>200</v>
       </c>
       <c r="F105" s="1" t="n">
         <v>0</v>
@@ -3902,7 +3914,7 @@
         <v>247</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C106" s="1" t="s">
         <v>248</v>
@@ -3911,7 +3923,7 @@
         <v>43</v>
       </c>
       <c r="E106" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F106" s="1" t="n">
         <v>0</v>
@@ -3922,7 +3934,7 @@
         <v>249</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>250</v>
@@ -3931,7 +3943,7 @@
         <v>43</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="F107" s="1" t="n">
         <v>0</v>
@@ -3942,7 +3954,7 @@
         <v>251</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>252</v>
@@ -3951,7 +3963,7 @@
         <v>43</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>242</v>
+        <v>204</v>
       </c>
       <c r="F108" s="1" t="n">
         <v>0</v>
@@ -3962,7 +3974,7 @@
         <v>253</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>254</v>
@@ -3971,7 +3983,7 @@
         <v>43</v>
       </c>
       <c r="E109" s="5" t="s">
-        <v>200</v>
+        <v>232</v>
       </c>
       <c r="F109" s="1" t="n">
         <v>0</v>
@@ -3982,7 +3994,7 @@
         <v>255</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>256</v>
@@ -3991,7 +4003,7 @@
         <v>43</v>
       </c>
       <c r="E110" s="5" t="s">
-        <v>200</v>
+        <v>246</v>
       </c>
       <c r="F110" s="1" t="n">
         <v>0</v>
@@ -4002,7 +4014,7 @@
         <v>257</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>258</v>
@@ -4011,7 +4023,7 @@
         <v>43</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="F111" s="1" t="n">
         <v>0</v>
@@ -4022,7 +4034,7 @@
         <v>259</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>260</v>
@@ -4031,7 +4043,7 @@
         <v>43</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>228</v>
+        <v>204</v>
       </c>
       <c r="F112" s="1" t="n">
         <v>0</v>
@@ -4042,7 +4054,7 @@
         <v>261</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>262</v>
@@ -4050,8 +4062,8 @@
       <c r="D113" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E113" s="9" t="s">
-        <v>263</v>
+      <c r="E113" s="5" t="s">
+        <v>204</v>
       </c>
       <c r="F113" s="1" t="n">
         <v>0</v>
@@ -4059,19 +4071,19 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="B114" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C114" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="B114" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C114" s="1" t="s">
-        <v>265</v>
-      </c>
       <c r="D114" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E114" s="9" t="s">
-        <v>266</v>
+      <c r="E114" s="5" t="s">
+        <v>232</v>
       </c>
       <c r="F114" s="1" t="n">
         <v>0</v>
@@ -4079,19 +4091,19 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="B115" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="D115" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E115" s="9" t="s">
         <v>267</v>
-      </c>
-      <c r="B115" s="6" t="s">
-        <v>194</v>
-      </c>
-      <c r="C115" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="D115" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E115" s="1" t="s">
-        <v>269</v>
       </c>
       <c r="F115" s="1" t="n">
         <v>0</v>
@@ -4099,19 +4111,19 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="B116" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="D116" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E116" s="9" t="s">
         <v>270</v>
-      </c>
-      <c r="B116" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C116" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="D116" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E116" s="1" t="s">
-        <v>269</v>
       </c>
       <c r="F116" s="1" t="n">
         <v>0</v>
@@ -4119,19 +4131,19 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="D117" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E117" s="1" t="s">
         <v>273</v>
-      </c>
-      <c r="B117" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C117" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="D117" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E117" s="1" t="s">
-        <v>269</v>
       </c>
       <c r="F117" s="1" t="n">
         <v>0</v>
@@ -4139,10 +4151,10 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B118" s="3" t="s">
         <v>275</v>
-      </c>
-      <c r="B118" s="3" t="s">
-        <v>271</v>
       </c>
       <c r="C118" s="1" t="s">
         <v>276</v>
@@ -4151,7 +4163,7 @@
         <v>43</v>
       </c>
       <c r="E118" s="1" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="F118" s="1" t="n">
         <v>0</v>
@@ -4159,19 +4171,19 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="B119" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C119" s="1" t="s">
         <v>278</v>
       </c>
-      <c r="B119" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C119" s="1" t="s">
-        <v>279</v>
-      </c>
       <c r="D119" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E119" s="7" t="s">
-        <v>280</v>
+      <c r="E119" s="1" t="s">
+        <v>273</v>
       </c>
       <c r="F119" s="1" t="n">
         <v>0</v>
@@ -4179,19 +4191,19 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
+        <v>279</v>
+      </c>
+      <c r="B120" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="D120" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E120" s="1" t="s">
         <v>281</v>
-      </c>
-      <c r="B120" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C120" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="D120" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E120" s="7" t="s">
-        <v>280</v>
       </c>
       <c r="F120" s="1" t="n">
         <v>0</v>
@@ -4199,19 +4211,19 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C121" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="B121" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C121" s="1" t="s">
+      <c r="D121" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E121" s="7" t="s">
         <v>284</v>
-      </c>
-      <c r="D121" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E121" s="7" t="s">
-        <v>280</v>
       </c>
       <c r="F121" s="1" t="n">
         <v>0</v>
@@ -4222,7 +4234,7 @@
         <v>285</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C122" s="1" t="s">
         <v>286</v>
@@ -4231,7 +4243,7 @@
         <v>43</v>
       </c>
       <c r="E122" s="7" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="F122" s="1" t="n">
         <v>0</v>
@@ -4239,19 +4251,19 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="3" t="s">
+        <v>287</v>
+      </c>
+      <c r="B123" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C123" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="B123" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C123" s="1" t="s">
-        <v>289</v>
-      </c>
       <c r="D123" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E123" s="7" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="F123" s="1" t="n">
         <v>0</v>
@@ -4259,19 +4271,19 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
+        <v>289</v>
+      </c>
+      <c r="B124" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C124" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="B124" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C124" s="1" t="s">
+      <c r="D124" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E124" s="7" t="s">
         <v>291</v>
-      </c>
-      <c r="D124" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E124" s="7" t="s">
-        <v>287</v>
       </c>
       <c r="F124" s="1" t="n">
         <v>0</v>
@@ -4282,7 +4294,7 @@
         <v>292</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>271</v>
+        <v>275</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>293</v>
@@ -4291,7 +4303,7 @@
         <v>43</v>
       </c>
       <c r="E125" s="7" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="F125" s="1" t="n">
         <v>0</v>
@@ -4299,19 +4311,19 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
+        <v>294</v>
+      </c>
+      <c r="B126" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C126" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="B126" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C126" s="1" t="s">
-        <v>296</v>
-      </c>
       <c r="D126" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E126" s="1" t="s">
-        <v>297</v>
+      <c r="E126" s="7" t="s">
+        <v>291</v>
       </c>
       <c r="F126" s="1" t="n">
         <v>0</v>
@@ -4319,19 +4331,19 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="3" t="s">
+        <v>296</v>
+      </c>
+      <c r="B127" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E127" s="7" t="s">
         <v>298</v>
-      </c>
-      <c r="B127" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C127" s="1" t="s">
-        <v>299</v>
-      </c>
-      <c r="D127" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E127" s="1" t="s">
-        <v>300</v>
       </c>
       <c r="F127" s="1" t="n">
         <v>0</v>
@@ -4339,19 +4351,19 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="D128" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E128" s="1" t="s">
         <v>301</v>
-      </c>
-      <c r="B128" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C128" s="1" t="s">
-        <v>302</v>
-      </c>
-      <c r="D128" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E128" s="1" t="s">
-        <v>303</v>
       </c>
       <c r="F128" s="1" t="n">
         <v>0</v>
@@ -4359,19 +4371,19 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="3" t="s">
+        <v>302</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="D129" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E129" s="1" t="s">
         <v>304</v>
-      </c>
-      <c r="B129" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C129" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="D129" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E129" s="1" t="s">
-        <v>306</v>
       </c>
       <c r="F129" s="1" t="n">
         <v>0</v>
@@ -4379,19 +4391,19 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
+        <v>305</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="D130" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E130" s="1" t="s">
         <v>307</v>
-      </c>
-      <c r="B130" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C130" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="D130" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E130" s="1" t="s">
-        <v>306</v>
       </c>
       <c r="F130" s="1" t="n">
         <v>0</v>
@@ -4399,19 +4411,19 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="3" t="s">
+        <v>308</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C131" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="B131" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="C131" s="1" t="s">
+      <c r="D131" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E131" s="1" t="s">
         <v>310</v>
-      </c>
-      <c r="D131" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E131" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="F131" s="1" t="n">
         <v>0</v>
@@ -4422,16 +4434,16 @@
         <v>311</v>
       </c>
       <c r="B132" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="C132" s="1" t="s">
         <v>312</v>
       </c>
-      <c r="C132" s="1" t="s">
-        <v>313</v>
-      </c>
       <c r="D132" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E132" s="1" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="F132" s="1" t="n">
         <v>0</v>
@@ -4439,19 +4451,19 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="3" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>312</v>
+        <v>275</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="D133" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E133" s="1" t="s">
-        <v>317</v>
+        <v>70</v>
       </c>
       <c r="F133" s="1" t="n">
         <v>0</v>
@@ -4459,16 +4471,19 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="B134" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="D134" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E134" s="1" t="s">
         <v>318</v>
-      </c>
-      <c r="B134" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="C134" s="1" t="s">
-        <v>319</v>
-      </c>
-      <c r="D134" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="F134" s="1" t="n">
         <v>0</v>
@@ -4476,67 +4491,64 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="3" t="s">
+        <v>319</v>
+      </c>
+      <c r="B135" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C135" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="B135" s="3" t="s">
-        <v>312</v>
-      </c>
-      <c r="C135" s="1" t="s">
+      <c r="D135" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E135" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="D135" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="F135" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A136" s="7" t="s">
+      <c r="A136" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="B136" s="7" t="s">
+      <c r="B136" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C136" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="C136" s="1" t="s">
+      <c r="D136" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F136" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A137" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="D136" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E136" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F136" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="7" t="s">
+      <c r="B137" s="3" t="s">
+        <v>316</v>
+      </c>
+      <c r="C137" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="B137" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C137" s="1" t="s">
+      <c r="D137" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F137" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A138" s="7" t="s">
         <v>326</v>
       </c>
-      <c r="D137" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E137" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F137" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="1" t="s">
+      <c r="B138" s="7" t="s">
         <v>327</v>
-      </c>
-      <c r="B138" s="7" t="s">
-        <v>323</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>328</v>
@@ -4545,27 +4557,27 @@
         <v>43</v>
       </c>
       <c r="E138" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F138" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A139" s="7" t="s">
         <v>329</v>
       </c>
-      <c r="F138" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="1" t="s">
+      <c r="B139" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C139" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="B139" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C139" s="1" t="s">
-        <v>331</v>
-      </c>
       <c r="D139" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E139" s="1" t="s">
-        <v>332</v>
+        <v>44</v>
       </c>
       <c r="F139" s="1" t="n">
         <v>0</v>
@@ -4573,19 +4585,19 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="B140" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="D140" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E140" s="1" t="s">
         <v>333</v>
-      </c>
-      <c r="B140" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C140" s="1" t="s">
-        <v>334</v>
-      </c>
-      <c r="D140" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E140" s="1" t="s">
-        <v>335</v>
       </c>
       <c r="F140" s="1" t="n">
         <v>0</v>
@@ -4593,36 +4605,39 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="B141" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="D141" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E141" s="1" t="s">
         <v>336</v>
       </c>
-      <c r="B141" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C141" s="1" t="s">
+      <c r="F141" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="D141" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F141" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A142" s="7" t="s">
+      <c r="B142" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C142" s="1" t="s">
         <v>338</v>
       </c>
-      <c r="B142" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C142" s="1" t="s">
+      <c r="D142" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E142" s="1" t="s">
         <v>339</v>
-      </c>
-      <c r="D142" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E142" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="F142" s="1" t="n">
         <v>0</v>
@@ -4633,7 +4648,7 @@
         <v>340</v>
       </c>
       <c r="B143" s="7" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>341</v>
@@ -4641,19 +4656,16 @@
       <c r="D143" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E143" s="1" t="s">
-        <v>100</v>
-      </c>
       <c r="F143" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A144" s="1" t="s">
+      <c r="A144" s="7" t="s">
         <v>342</v>
       </c>
       <c r="B144" s="7" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>343</v>
@@ -4662,7 +4674,7 @@
         <v>43</v>
       </c>
       <c r="E144" s="1" t="s">
-        <v>185</v>
+        <v>70</v>
       </c>
       <c r="F144" s="1" t="n">
         <v>0</v>
@@ -4673,7 +4685,7 @@
         <v>344</v>
       </c>
       <c r="B145" s="7" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>345</v>
@@ -4682,7 +4694,7 @@
         <v>43</v>
       </c>
       <c r="E145" s="1" t="s">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="F145" s="1" t="n">
         <v>0</v>
@@ -4692,8 +4704,8 @@
       <c r="A146" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="B146" s="1" t="s">
-        <v>323</v>
+      <c r="B146" s="7" t="s">
+        <v>327</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>347</v>
@@ -4702,7 +4714,10 @@
         <v>43</v>
       </c>
       <c r="E146" s="1" t="s">
-        <v>332</v>
+        <v>189</v>
+      </c>
+      <c r="F146" s="1" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4710,7 +4725,7 @@
         <v>348</v>
       </c>
       <c r="B147" s="7" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>349</v>
@@ -4719,7 +4734,7 @@
         <v>43</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>44</v>
+        <v>150</v>
       </c>
       <c r="F147" s="1" t="n">
         <v>0</v>
@@ -4729,8 +4744,8 @@
       <c r="A148" s="1" t="s">
         <v>350</v>
       </c>
-      <c r="B148" s="7" t="s">
-        <v>323</v>
+      <c r="B148" s="1" t="s">
+        <v>327</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>351</v>
@@ -4739,10 +4754,7 @@
         <v>43</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F148" s="1" t="n">
-        <v>0</v>
+        <v>336</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4750,7 +4762,7 @@
         <v>352</v>
       </c>
       <c r="B149" s="7" t="s">
-        <v>323</v>
+        <v>327</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>353</v>
@@ -4759,7 +4771,7 @@
         <v>43</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>354</v>
+        <v>44</v>
       </c>
       <c r="F149" s="1" t="n">
         <v>0</v>
@@ -4767,19 +4779,19 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="B150" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C150" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="B150" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C150" s="1" t="s">
-        <v>356</v>
-      </c>
       <c r="D150" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E150" s="1" t="s">
-        <v>150</v>
+        <v>44</v>
       </c>
       <c r="F150" s="1" t="n">
         <v>0</v>
@@ -4787,19 +4799,19 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="B151" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C151" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="B151" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C151" s="1" t="s">
+      <c r="D151" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E151" s="1" t="s">
         <v>358</v>
-      </c>
-      <c r="D151" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E151" s="1" t="s">
-        <v>70</v>
       </c>
       <c r="F151" s="1" t="n">
         <v>0</v>
@@ -4810,16 +4822,16 @@
         <v>359</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C152" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C152" s="1" t="s">
         <v>360</v>
       </c>
       <c r="D152" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E152" s="1" t="s">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="F152" s="1" t="n">
         <v>0</v>
@@ -4830,9 +4842,9 @@
         <v>361</v>
       </c>
       <c r="B153" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C153" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C153" s="1" t="s">
         <v>362</v>
       </c>
       <c r="D153" s="1" t="s">
@@ -4850,16 +4862,16 @@
         <v>363</v>
       </c>
       <c r="B154" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C154" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="C154" s="7" t="s">
         <v>364</v>
       </c>
       <c r="D154" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E154" s="1" t="s">
-        <v>354</v>
+        <v>70</v>
       </c>
       <c r="F154" s="1" t="n">
         <v>0</v>
@@ -4870,23 +4882,61 @@
         <v>365</v>
       </c>
       <c r="B155" s="7" t="s">
-        <v>323</v>
-      </c>
-      <c r="C155" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="C155" s="7" t="s">
         <v>366</v>
       </c>
       <c r="D155" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E155" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F155" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="B156" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C156" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="D156" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E156" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="F156" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="B157" s="7" t="s">
+        <v>327</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="D157" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E157" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F155" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="1048575" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="F157" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
value fixed in SpParamsDefinition
</commit_message>
<xml_diff>
--- a/data-raw/SpParamsDefinition.xlsx
+++ b/data-raw/SpParamsDefinition.xlsx
@@ -1904,7 +1904,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="70.17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.31"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.35"/>
   </cols>
   <sheetData>
@@ -3651,7 +3651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="17.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
         <v>216</v>
       </c>
@@ -4755,6 +4755,9 @@
       </c>
       <c r="E148" s="1" t="s">
         <v>336</v>
+      </c>
+      <c r="F148" s="0" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
New parameter names for Baldocchi and Jarvis
</commit_message>
<xml_diff>
--- a/data-raw/SpParamsDefinition.xlsx
+++ b/data-raw/SpParamsDefinition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="376">
   <si>
     <t xml:space="preserve">ParameterName</t>
   </si>
@@ -481,13 +481,19 @@
     <t xml:space="preserve">Minimum fuel moisture (in percent of dry weight)</t>
   </si>
   <si>
+    <t xml:space="preserve">Ptlp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leaf water potential at turgor loss point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mpa</t>
+  </si>
+  <si>
     <t xml:space="preserve">LeafPI0</t>
   </si>
   <si>
     <t xml:space="preserve">Osmotic potential at full turgor of leaves</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mpa</t>
   </si>
   <si>
     <t xml:space="preserve">LeafEPS</t>
@@ -788,7 +794,73 @@
     <t xml:space="preserve">Maximum stomatal conductance to water vapour</t>
   </si>
   <si>
-    <t xml:space="preserve">Gsw_AC_slope</t>
+    <t xml:space="preserve">Gsw_Toptim_Jarvis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Temperature corresponding to maximal stomatal conductance (Jarvis stomatal model)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Gsw_Tsens</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">_Jarvis</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Stomatal sensitivity to temperature</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> (Jarvis stomatal model)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Gsw_AC_slope</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">_Baldocchi</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Slope of the Gsw vs Ac/Cs relationship (Baldocchi model).</t>
@@ -869,28 +941,70 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Gs_Toptim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Temperature corresponding to maximal stomatal conductance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gs_Tsens</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stomatal sensitivity to temperature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gs_P50</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Water potential causing 50% reduction in stomatal conductance</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gs_slope</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rate of decrease in stomatal conductance at Gs_P50</t>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Gsw_P50</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">_Baldocchi</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Water potential causing 50% reduction in stomatal conductance (Baldocchi stomatal model)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Gsw_slope</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">_Baldocchi</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Rate of decrease in stomatal conductance at Gsw_Baldocchi_P50 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">(Baldocchi stomatal model)</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">%/MPa</t>
@@ -1616,7 +1730,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* \-??\ _€_-;_-@_-"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -1677,6 +1791,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1778,7 +1898,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1907,10 +2027,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F158"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultColWidth="10.25" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="21.13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="70.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.32"/>
@@ -3206,7 +3326,7 @@
         <v>43</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F69" s="1" t="n">
         <v>0</v>
@@ -3226,7 +3346,7 @@
         <v>43</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F70" s="1" t="n">
         <v>0</v>
@@ -3266,7 +3386,7 @@
         <v>43</v>
       </c>
       <c r="E72" s="5" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F72" s="1" t="n">
         <v>0</v>
@@ -3277,16 +3397,16 @@
         <v>166</v>
       </c>
       <c r="B73" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="C73" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="C73" s="1" t="s">
-        <v>168</v>
-      </c>
       <c r="D73" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E73" s="5" t="s">
-        <v>169</v>
+        <v>150</v>
       </c>
       <c r="F73" s="1" t="n">
         <v>0</v>
@@ -3294,19 +3414,19 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="C74" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="B74" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C74" s="1" t="s">
+      <c r="D74" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E74" s="5" t="s">
         <v>171</v>
-      </c>
-      <c r="D74" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E74" s="5" t="s">
-        <v>172</v>
       </c>
       <c r="F74" s="1" t="n">
         <v>0</v>
@@ -3314,19 +3434,19 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>173</v>
       </c>
-      <c r="B75" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="C75" s="1" t="s">
+      <c r="D75" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E75" s="5" t="s">
         <v>174</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E75" s="5" t="s">
-        <v>150</v>
       </c>
       <c r="F75" s="1" t="n">
         <v>0</v>
@@ -3337,7 +3457,7 @@
         <v>175</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>176</v>
@@ -3357,7 +3477,7 @@
         <v>177</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C77" s="1" t="s">
         <v>178</v>
@@ -3377,16 +3497,16 @@
         <v>179</v>
       </c>
       <c r="B78" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>180</v>
       </c>
-      <c r="C78" s="1" t="s">
-        <v>181</v>
-      </c>
       <c r="D78" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E78" s="5" t="s">
-        <v>182</v>
+        <v>150</v>
       </c>
       <c r="F78" s="1" t="n">
         <v>0</v>
@@ -3394,19 +3514,19 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C79" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="B79" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="C79" s="1" t="s">
+      <c r="D79" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E79" s="5" t="s">
         <v>184</v>
-      </c>
-      <c r="D79" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E79" s="5" t="s">
-        <v>182</v>
       </c>
       <c r="F79" s="1" t="n">
         <v>0</v>
@@ -3417,7 +3537,7 @@
         <v>185</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C80" s="1" t="s">
         <v>186</v>
@@ -3426,7 +3546,7 @@
         <v>43</v>
       </c>
       <c r="E80" s="5" t="s">
-        <v>70</v>
+        <v>184</v>
       </c>
       <c r="F80" s="1" t="n">
         <v>0</v>
@@ -3437,7 +3557,7 @@
         <v>187</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C81" s="1" t="s">
         <v>188</v>
@@ -3446,7 +3566,7 @@
         <v>43</v>
       </c>
       <c r="E81" s="5" t="s">
-        <v>189</v>
+        <v>70</v>
       </c>
       <c r="F81" s="1" t="n">
         <v>0</v>
@@ -3454,19 +3574,19 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C82" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="B82" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="C82" s="1" t="s">
+      <c r="D82" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E82" s="5" t="s">
         <v>191</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E82" s="5" t="s">
-        <v>189</v>
       </c>
       <c r="F82" s="1" t="n">
         <v>0</v>
@@ -3477,7 +3597,7 @@
         <v>192</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C83" s="1" t="s">
         <v>193</v>
@@ -3486,7 +3606,7 @@
         <v>43</v>
       </c>
       <c r="E83" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F83" s="1" t="n">
         <v>0</v>
@@ -3497,7 +3617,7 @@
         <v>194</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C84" s="1" t="s">
         <v>195</v>
@@ -3506,7 +3626,7 @@
         <v>43</v>
       </c>
       <c r="E84" s="5" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="F84" s="1" t="n">
         <v>0</v>
@@ -3514,28 +3634,30 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B85" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="C85" s="1" t="s">
         <v>197</v>
       </c>
-      <c r="B85" s="6" t="s">
+      <c r="D85" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E85" s="5" t="s">
         <v>198</v>
       </c>
-      <c r="C85" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E85" s="5"/>
       <c r="F85" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
+        <v>199</v>
+      </c>
+      <c r="B86" s="6" t="s">
         <v>200</v>
-      </c>
-      <c r="B86" s="6" t="s">
-        <v>198</v>
       </c>
       <c r="C86" s="1" t="s">
         <v>201</v>
@@ -3553,7 +3675,7 @@
         <v>202</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C87" s="1" t="s">
         <v>203</v>
@@ -3561,27 +3683,27 @@
       <c r="D87" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E87" s="5" t="s">
-        <v>204</v>
-      </c>
+      <c r="E87" s="5"/>
       <c r="F87" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C88" s="1" t="s">
         <v>205</v>
       </c>
-      <c r="B88" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C88" s="1" t="s">
+      <c r="D88" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E88" s="5" t="s">
         <v>206</v>
       </c>
-      <c r="D88" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E88" s="5"/>
       <c r="F88" s="1" t="n">
         <v>0</v>
       </c>
@@ -3591,7 +3713,7 @@
         <v>207</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C89" s="1" t="s">
         <v>208</v>
@@ -3599,27 +3721,27 @@
       <c r="D89" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E89" s="5" t="s">
-        <v>209</v>
-      </c>
+      <c r="E89" s="5"/>
       <c r="F89" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="B90" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C90" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="B90" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C90" s="1" t="s">
+      <c r="D90" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E90" s="5" t="s">
         <v>211</v>
       </c>
-      <c r="D90" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E90" s="5"/>
       <c r="F90" s="1" t="n">
         <v>0</v>
       </c>
@@ -3629,7 +3751,7 @@
         <v>212</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C91" s="1" t="s">
         <v>213</v>
@@ -3647,7 +3769,7 @@
         <v>214</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C92" s="1" t="s">
         <v>215</v>
@@ -3660,41 +3782,39 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
         <v>216</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C93" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="C93" s="1" t="s">
         <v>217</v>
       </c>
       <c r="D93" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E93" s="5" t="s">
+      <c r="E93" s="5"/>
+      <c r="F93" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="F93" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A94" s="3" t="s">
+      <c r="B94" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C94" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="B94" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C94" s="1" t="s">
+      <c r="D94" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E94" s="5" t="s">
         <v>220</v>
-      </c>
-      <c r="D94" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E94" s="5" t="s">
-        <v>218</v>
       </c>
       <c r="F94" s="1" t="n">
         <v>0</v>
@@ -3705,7 +3825,7 @@
         <v>221</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C95" s="1" t="s">
         <v>222</v>
@@ -3714,7 +3834,7 @@
         <v>43</v>
       </c>
       <c r="E95" s="5" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="F95" s="1" t="n">
         <v>0</v>
@@ -3722,13 +3842,13 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="B96" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C96" s="1" t="s">
         <v>224</v>
-      </c>
-      <c r="B96" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C96" s="1" t="s">
-        <v>225</v>
       </c>
       <c r="D96" s="1" t="s">
         <v>43</v>
@@ -3740,15 +3860,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="B97" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C97" s="1" t="s">
         <v>226</v>
-      </c>
-      <c r="B97" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C97" s="1" t="s">
-        <v>227</v>
       </c>
       <c r="D97" s="1" t="s">
         <v>43</v>
@@ -3758,32 +3878,32 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="B98" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C98" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="B98" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C98" s="1" t="s">
+      <c r="D98" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E98" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="D98" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E98" s="5" t="s">
-        <v>204</v>
-      </c>
       <c r="F98" s="1" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
         <v>230</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C99" s="1" t="s">
         <v>231</v>
@@ -3792,27 +3912,27 @@
         <v>43</v>
       </c>
       <c r="E99" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="F99" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A100" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="F99" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A100" s="3" t="s">
+      <c r="B100" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C100" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="B100" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C100" s="1" t="s">
+      <c r="D100" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E100" s="5" t="s">
         <v>234</v>
-      </c>
-      <c r="D100" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E100" s="5" t="s">
-        <v>235</v>
       </c>
       <c r="F100" s="1" t="n">
         <v>0</v>
@@ -3820,19 +3940,19 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="B101" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>236</v>
       </c>
-      <c r="B101" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C101" s="1" t="s">
+      <c r="D101" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E101" s="5" t="s">
         <v>237</v>
-      </c>
-      <c r="D101" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E101" s="5" t="s">
-        <v>204</v>
       </c>
       <c r="F101" s="1" t="n">
         <v>0</v>
@@ -3843,7 +3963,7 @@
         <v>238</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C102" s="1" t="s">
         <v>239</v>
@@ -3852,7 +3972,7 @@
         <v>43</v>
       </c>
       <c r="E102" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F102" s="1" t="n">
         <v>0</v>
@@ -3863,7 +3983,7 @@
         <v>240</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C103" s="1" t="s">
         <v>241</v>
@@ -3872,7 +3992,7 @@
         <v>43</v>
       </c>
       <c r="E103" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F103" s="1" t="n">
         <v>0</v>
@@ -3883,7 +4003,7 @@
         <v>242</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C104" s="1" t="s">
         <v>243</v>
@@ -3892,7 +4012,7 @@
         <v>43</v>
       </c>
       <c r="E104" s="5" t="s">
-        <v>232</v>
+        <v>206</v>
       </c>
       <c r="F104" s="1" t="n">
         <v>0</v>
@@ -3903,7 +4023,7 @@
         <v>244</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C105" s="1" t="s">
         <v>245</v>
@@ -3912,7 +4032,7 @@
         <v>43</v>
       </c>
       <c r="E105" s="5" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="F105" s="1" t="n">
         <v>0</v>
@@ -3920,19 +4040,19 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="B106" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C106" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="B106" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C106" s="1" t="s">
+      <c r="D106" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E106" s="5" t="s">
         <v>248</v>
-      </c>
-      <c r="D106" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E106" s="5" t="s">
-        <v>204</v>
       </c>
       <c r="F106" s="1" t="n">
         <v>0</v>
@@ -3943,7 +4063,7 @@
         <v>249</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C107" s="1" t="s">
         <v>250</v>
@@ -3952,7 +4072,7 @@
         <v>43</v>
       </c>
       <c r="E107" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F107" s="1" t="n">
         <v>0</v>
@@ -3963,7 +4083,7 @@
         <v>251</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C108" s="1" t="s">
         <v>252</v>
@@ -3972,7 +4092,7 @@
         <v>43</v>
       </c>
       <c r="E108" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F108" s="1" t="n">
         <v>0</v>
@@ -3983,7 +4103,7 @@
         <v>253</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C109" s="1" t="s">
         <v>254</v>
@@ -3992,7 +4112,7 @@
         <v>43</v>
       </c>
       <c r="E109" s="5" t="s">
-        <v>232</v>
+        <v>206</v>
       </c>
       <c r="F109" s="1" t="n">
         <v>0</v>
@@ -4003,7 +4123,7 @@
         <v>255</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C110" s="1" t="s">
         <v>256</v>
@@ -4012,7 +4132,7 @@
         <v>43</v>
       </c>
       <c r="E110" s="5" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="F110" s="1" t="n">
         <v>0</v>
@@ -4023,7 +4143,7 @@
         <v>257</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C111" s="1" t="s">
         <v>258</v>
@@ -4032,7 +4152,7 @@
         <v>43</v>
       </c>
       <c r="E111" s="5" t="s">
-        <v>204</v>
+        <v>248</v>
       </c>
       <c r="F111" s="1" t="n">
         <v>0</v>
@@ -4043,7 +4163,7 @@
         <v>259</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C112" s="1" t="s">
         <v>260</v>
@@ -4052,7 +4172,7 @@
         <v>43</v>
       </c>
       <c r="E112" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F112" s="1" t="n">
         <v>0</v>
@@ -4063,7 +4183,7 @@
         <v>261</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C113" s="1" t="s">
         <v>262</v>
@@ -4072,7 +4192,7 @@
         <v>43</v>
       </c>
       <c r="E113" s="5" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F113" s="1" t="n">
         <v>0</v>
@@ -4083,7 +4203,7 @@
         <v>263</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C114" s="1" t="s">
         <v>264</v>
@@ -4092,7 +4212,7 @@
         <v>43</v>
       </c>
       <c r="E114" s="5" t="s">
-        <v>232</v>
+        <v>206</v>
       </c>
       <c r="F114" s="1" t="n">
         <v>0</v>
@@ -4103,7 +4223,7 @@
         <v>265</v>
       </c>
       <c r="B115" s="6" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C115" s="1" t="s">
         <v>266</v>
@@ -4111,8 +4231,8 @@
       <c r="D115" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E115" s="9" t="s">
-        <v>267</v>
+      <c r="E115" s="5" t="s">
+        <v>234</v>
       </c>
       <c r="F115" s="1" t="n">
         <v>0</v>
@@ -4120,19 +4240,19 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="B116" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C116" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="B116" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C116" s="1" t="s">
+      <c r="D116" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E116" s="9" t="s">
         <v>269</v>
-      </c>
-      <c r="D116" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E116" s="9" t="s">
-        <v>270</v>
       </c>
       <c r="F116" s="1" t="n">
         <v>0</v>
@@ -4140,19 +4260,19 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="B117" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C117" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="B117" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="C117" s="1" t="s">
+      <c r="D117" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E117" s="9" t="s">
         <v>272</v>
-      </c>
-      <c r="D117" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E117" s="1" t="s">
-        <v>273</v>
       </c>
       <c r="F117" s="1" t="n">
         <v>0</v>
@@ -4160,19 +4280,19 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B118" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C118" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="B118" s="3" t="s">
+      <c r="D118" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E118" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="C118" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="D118" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E118" s="1" t="s">
-        <v>273</v>
       </c>
       <c r="F118" s="1" t="n">
         <v>0</v>
@@ -4180,10 +4300,10 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="B119" s="3" t="s">
         <v>277</v>
-      </c>
-      <c r="B119" s="3" t="s">
-        <v>275</v>
       </c>
       <c r="C119" s="1" t="s">
         <v>278</v>
@@ -4192,7 +4312,7 @@
         <v>43</v>
       </c>
       <c r="E119" s="1" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="F119" s="1" t="n">
         <v>0</v>
@@ -4203,7 +4323,7 @@
         <v>279</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C120" s="1" t="s">
         <v>280</v>
@@ -4212,7 +4332,7 @@
         <v>43</v>
       </c>
       <c r="E120" s="1" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F120" s="1" t="n">
         <v>0</v>
@@ -4220,19 +4340,19 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B121" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C121" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="B121" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C121" s="1" t="s">
+      <c r="D121" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E121" s="1" t="s">
         <v>283</v>
-      </c>
-      <c r="D121" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E121" s="7" t="s">
-        <v>284</v>
       </c>
       <c r="F121" s="1" t="n">
         <v>0</v>
@@ -4240,19 +4360,19 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="B122" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C122" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="B122" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C122" s="1" t="s">
+      <c r="D122" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E122" s="7" t="s">
         <v>286</v>
-      </c>
-      <c r="D122" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E122" s="7" t="s">
-        <v>284</v>
       </c>
       <c r="F122" s="1" t="n">
         <v>0</v>
@@ -4263,7 +4383,7 @@
         <v>287</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>288</v>
@@ -4272,7 +4392,7 @@
         <v>43</v>
       </c>
       <c r="E123" s="7" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F123" s="1" t="n">
         <v>0</v>
@@ -4283,7 +4403,7 @@
         <v>289</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>290</v>
@@ -4292,7 +4412,7 @@
         <v>43</v>
       </c>
       <c r="E124" s="7" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="F124" s="1" t="n">
         <v>0</v>
@@ -4300,19 +4420,19 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="3" t="s">
+        <v>291</v>
+      </c>
+      <c r="B125" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C125" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="B125" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C125" s="1" t="s">
+      <c r="D125" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E125" s="7" t="s">
         <v>293</v>
-      </c>
-      <c r="D125" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E125" s="7" t="s">
-        <v>291</v>
       </c>
       <c r="F125" s="1" t="n">
         <v>0</v>
@@ -4323,7 +4443,7 @@
         <v>294</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>295</v>
@@ -4332,7 +4452,7 @@
         <v>43</v>
       </c>
       <c r="E126" s="7" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F126" s="1" t="n">
         <v>0</v>
@@ -4343,7 +4463,7 @@
         <v>296</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>297</v>
@@ -4352,7 +4472,7 @@
         <v>43</v>
       </c>
       <c r="E127" s="7" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="F127" s="1" t="n">
         <v>0</v>
@@ -4360,19 +4480,19 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
+        <v>298</v>
+      </c>
+      <c r="B128" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C128" s="1" t="s">
         <v>299</v>
       </c>
-      <c r="B128" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C128" s="1" t="s">
+      <c r="D128" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E128" s="7" t="s">
         <v>300</v>
-      </c>
-      <c r="D128" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E128" s="1" t="s">
-        <v>301</v>
       </c>
       <c r="F128" s="1" t="n">
         <v>0</v>
@@ -4380,19 +4500,19 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="B129" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C129" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="B129" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C129" s="1" t="s">
+      <c r="D129" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E129" s="1" t="s">
         <v>303</v>
-      </c>
-      <c r="D129" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E129" s="1" t="s">
-        <v>304</v>
       </c>
       <c r="F129" s="1" t="n">
         <v>0</v>
@@ -4400,19 +4520,19 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="B130" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C130" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="B130" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C130" s="1" t="s">
+      <c r="D130" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E130" s="1" t="s">
         <v>306</v>
-      </c>
-      <c r="D130" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E130" s="1" t="s">
-        <v>307</v>
       </c>
       <c r="F130" s="1" t="n">
         <v>0</v>
@@ -4420,19 +4540,19 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="3" t="s">
+        <v>307</v>
+      </c>
+      <c r="B131" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C131" s="1" t="s">
         <v>308</v>
       </c>
-      <c r="B131" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C131" s="1" t="s">
+      <c r="D131" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E131" s="1" t="s">
         <v>309</v>
-      </c>
-      <c r="D131" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E131" s="1" t="s">
-        <v>310</v>
       </c>
       <c r="F131" s="1" t="n">
         <v>0</v>
@@ -4440,19 +4560,19 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
+        <v>310</v>
+      </c>
+      <c r="B132" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C132" s="1" t="s">
         <v>311</v>
       </c>
-      <c r="B132" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C132" s="1" t="s">
+      <c r="D132" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E132" s="1" t="s">
         <v>312</v>
-      </c>
-      <c r="D132" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E132" s="1" t="s">
-        <v>313</v>
       </c>
       <c r="F132" s="1" t="n">
         <v>0</v>
@@ -4460,19 +4580,19 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="B133" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C133" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="B133" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C133" s="1" t="s">
+      <c r="D133" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E133" s="1" t="s">
         <v>315</v>
-      </c>
-      <c r="D133" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E133" s="1" t="s">
-        <v>313</v>
       </c>
       <c r="F133" s="1" t="n">
         <v>0</v>
@@ -4483,7 +4603,7 @@
         <v>316</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>317</v>
@@ -4492,7 +4612,7 @@
         <v>43</v>
       </c>
       <c r="E134" s="1" t="s">
-        <v>70</v>
+        <v>315</v>
       </c>
       <c r="F134" s="1" t="n">
         <v>0</v>
@@ -4503,16 +4623,16 @@
         <v>318</v>
       </c>
       <c r="B135" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="C135" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="C135" s="1" t="s">
-        <v>320</v>
-      </c>
       <c r="D135" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E135" s="1" t="s">
-        <v>321</v>
+        <v>70</v>
       </c>
       <c r="F135" s="1" t="n">
         <v>0</v>
@@ -4520,19 +4640,19 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
+        <v>320</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C136" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="B136" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="C136" s="1" t="s">
+      <c r="D136" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E136" s="1" t="s">
         <v>323</v>
-      </c>
-      <c r="D136" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E136" s="1" t="s">
-        <v>324</v>
       </c>
       <c r="F136" s="1" t="n">
         <v>0</v>
@@ -4540,16 +4660,19 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="3" t="s">
+        <v>324</v>
+      </c>
+      <c r="B137" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C137" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="B137" s="3" t="s">
-        <v>319</v>
-      </c>
-      <c r="C137" s="1" t="s">
+      <c r="D137" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E137" s="1" t="s">
         <v>326</v>
-      </c>
-      <c r="D137" s="1" t="s">
-        <v>43</v>
       </c>
       <c r="F137" s="1" t="n">
         <v>0</v>
@@ -4560,7 +4683,7 @@
         <v>327</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C138" s="1" t="s">
         <v>328</v>
@@ -4573,20 +4696,17 @@
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="7" t="s">
+      <c r="A139" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="B139" s="7" t="s">
+      <c r="B139" s="3" t="s">
+        <v>321</v>
+      </c>
+      <c r="C139" s="1" t="s">
         <v>330</v>
       </c>
-      <c r="C139" s="1" t="s">
-        <v>331</v>
-      </c>
       <c r="D139" s="1" t="s">
         <v>43</v>
-      </c>
-      <c r="E139" s="1" t="s">
-        <v>44</v>
       </c>
       <c r="F139" s="1" t="n">
         <v>0</v>
@@ -4594,10 +4714,10 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="B140" s="7" t="s">
         <v>332</v>
-      </c>
-      <c r="B140" s="7" t="s">
-        <v>330</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>333</v>
@@ -4613,11 +4733,11 @@
       </c>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A141" s="1" t="s">
+      <c r="A141" s="7" t="s">
         <v>334</v>
       </c>
       <c r="B141" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>335</v>
@@ -4626,7 +4746,7 @@
         <v>43</v>
       </c>
       <c r="E141" s="1" t="s">
-        <v>336</v>
+        <v>44</v>
       </c>
       <c r="F141" s="1" t="n">
         <v>0</v>
@@ -4634,19 +4754,19 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="B142" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="C142" s="1" t="s">
         <v>337</v>
       </c>
-      <c r="B142" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="C142" s="1" t="s">
+      <c r="D142" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E142" s="1" t="s">
         <v>338</v>
-      </c>
-      <c r="D142" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E142" s="1" t="s">
-        <v>339</v>
       </c>
       <c r="F142" s="1" t="n">
         <v>0</v>
@@ -4654,19 +4774,19 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="B143" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="C143" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="B143" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="C143" s="1" t="s">
+      <c r="D143" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E143" s="1" t="s">
         <v>341</v>
-      </c>
-      <c r="D143" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E143" s="1" t="s">
-        <v>342</v>
       </c>
       <c r="F143" s="1" t="n">
         <v>0</v>
@@ -4674,27 +4794,30 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="B144" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="C144" s="1" t="s">
         <v>343</v>
       </c>
-      <c r="B144" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="C144" s="1" t="s">
+      <c r="D144" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E144" s="1" t="s">
         <v>344</v>
       </c>
-      <c r="D144" s="1" t="s">
-        <v>43</v>
-      </c>
       <c r="F144" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A145" s="7" t="s">
+      <c r="A145" s="1" t="s">
         <v>345</v>
       </c>
       <c r="B145" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>346</v>
@@ -4702,19 +4825,16 @@
       <c r="D145" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="E145" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="F145" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="1" t="s">
+      <c r="A146" s="7" t="s">
         <v>347</v>
       </c>
       <c r="B146" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>348</v>
@@ -4723,7 +4843,7 @@
         <v>43</v>
       </c>
       <c r="E146" s="1" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="F146" s="1" t="n">
         <v>0</v>
@@ -4734,7 +4854,7 @@
         <v>349</v>
       </c>
       <c r="B147" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>350</v>
@@ -4743,7 +4863,7 @@
         <v>43</v>
       </c>
       <c r="E147" s="1" t="s">
-        <v>189</v>
+        <v>100</v>
       </c>
       <c r="F147" s="1" t="n">
         <v>0</v>
@@ -4754,7 +4874,7 @@
         <v>351</v>
       </c>
       <c r="B148" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>352</v>
@@ -4763,7 +4883,7 @@
         <v>43</v>
       </c>
       <c r="E148" s="1" t="s">
-        <v>150</v>
+        <v>191</v>
       </c>
       <c r="F148" s="1" t="n">
         <v>0</v>
@@ -4773,8 +4893,8 @@
       <c r="A149" s="1" t="s">
         <v>353</v>
       </c>
-      <c r="B149" s="1" t="s">
-        <v>330</v>
+      <c r="B149" s="7" t="s">
+        <v>332</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>354</v>
@@ -4783,7 +4903,7 @@
         <v>43</v>
       </c>
       <c r="E149" s="1" t="s">
-        <v>339</v>
+        <v>150</v>
       </c>
       <c r="F149" s="1" t="n">
         <v>0</v>
@@ -4793,8 +4913,8 @@
       <c r="A150" s="1" t="s">
         <v>355</v>
       </c>
-      <c r="B150" s="7" t="s">
-        <v>330</v>
+      <c r="B150" s="1" t="s">
+        <v>332</v>
       </c>
       <c r="C150" s="1" t="s">
         <v>356</v>
@@ -4803,7 +4923,7 @@
         <v>43</v>
       </c>
       <c r="E150" s="1" t="s">
-        <v>44</v>
+        <v>341</v>
       </c>
       <c r="F150" s="1" t="n">
         <v>0</v>
@@ -4814,7 +4934,7 @@
         <v>357</v>
       </c>
       <c r="B151" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>358</v>
@@ -4834,7 +4954,7 @@
         <v>359</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>360</v>
@@ -4843,7 +4963,7 @@
         <v>43</v>
       </c>
       <c r="E152" s="1" t="s">
-        <v>361</v>
+        <v>44</v>
       </c>
       <c r="F152" s="1" t="n">
         <v>0</v>
@@ -4851,19 +4971,19 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="B153" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="C153" s="1" t="s">
         <v>362</v>
       </c>
-      <c r="B153" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="C153" s="1" t="s">
+      <c r="D153" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E153" s="1" t="s">
         <v>363</v>
-      </c>
-      <c r="D153" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E153" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="F153" s="1" t="n">
         <v>0</v>
@@ -4874,7 +4994,7 @@
         <v>364</v>
       </c>
       <c r="B154" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>365</v>
@@ -4883,7 +5003,7 @@
         <v>43</v>
       </c>
       <c r="E154" s="1" t="s">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="F154" s="1" t="n">
         <v>0</v>
@@ -4894,9 +5014,9 @@
         <v>366</v>
       </c>
       <c r="B155" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="C155" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="C155" s="1" t="s">
         <v>367</v>
       </c>
       <c r="D155" s="1" t="s">
@@ -4914,7 +5034,7 @@
         <v>368</v>
       </c>
       <c r="B156" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C156" s="7" t="s">
         <v>369</v>
@@ -4934,16 +5054,16 @@
         <v>370</v>
       </c>
       <c r="B157" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="C157" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="C157" s="7" t="s">
         <v>371</v>
       </c>
       <c r="D157" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E157" s="1" t="s">
-        <v>361</v>
+        <v>70</v>
       </c>
       <c r="F157" s="1" t="n">
         <v>0</v>
@@ -4954,7 +5074,7 @@
         <v>372</v>
       </c>
       <c r="B158" s="7" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>373</v>
@@ -4963,12 +5083,33 @@
         <v>43</v>
       </c>
       <c r="E158" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="F158" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A159" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="B159" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="D159" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E159" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F158" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
+      <c r="F159" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
update definitions and params
</commit_message>
<xml_diff>
--- a/data-raw/SpParamsDefinition.xlsx
+++ b/data-raw/SpParamsDefinition.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="757" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="378">
   <si>
     <t xml:space="preserve">ParameterName</t>
   </si>
@@ -800,67 +800,13 @@
     <t xml:space="preserve">Temperature corresponding to maximal stomatal conductance (Jarvis stomatal model)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Gsw_Tsens</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">_Jarvis</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Stomatal sensitivity to temperature</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> (Jarvis stomatal model)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Gsw_AC_slope</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">_Baldocchi</t>
-    </r>
+    <t xml:space="preserve">Gsw_Tsens_Jarvis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stomatal sensitivity to temperature (Jarvis stomatal model)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gsw_AC_slope_Baldocchi</t>
   </si>
   <si>
     <t xml:space="preserve">Slope of the Gsw vs Ac/Cs relationship (Baldocchi model).</t>
@@ -941,70 +887,16 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Gsw_P50</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">_Baldocchi</t>
-    </r>
+    <t xml:space="preserve">Gsw_P50_Baldocchi</t>
   </si>
   <si>
     <t xml:space="preserve">Water potential causing 50% reduction in stomatal conductance (Baldocchi stomatal model)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Gsw_slope</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">_Baldocchi</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Rate of decrease in stomatal conductance at Gsw_Baldocchi_P50 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">(Baldocchi stomatal model)</t>
-    </r>
+    <t xml:space="preserve">Gsw_slope_Baldocchi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rate of decrease in stomatal conductance at Gsw_Baldocchi_P50 (Baldocchi stomatal model)</t>
   </si>
   <si>
     <t xml:space="preserve">%/MPa</t>
@@ -1665,6 +1557,12 @@
     <t xml:space="preserve">Age of recruiment</t>
   </si>
   <si>
+    <t xml:space="preserve">RecrTreeDBH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recruitment tree (sapling) stem diameter at breast height</t>
+  </si>
+  <si>
     <t xml:space="preserve">RecrTreeHeight</t>
   </si>
   <si>
@@ -1730,7 +1628,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ _€_-;\-* #,##0.00\ _€_-;_-* \-??\ _€_-;_-@_-"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -1791,12 +1689,6 @@
       <name val="Times New Roman"/>
       <family val="1"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
@@ -1898,7 +1790,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2027,10 +1919,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F1048576"/>
+  <dimension ref="A1:F160"/>
   <sheetFormatPr defaultColWidth="10.25" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="70.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11.32"/>
@@ -3860,7 +3752,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
         <v>225</v>
       </c>
@@ -3878,7 +3770,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
         <v>227</v>
       </c>
@@ -3898,7 +3790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
         <v>230</v>
       </c>
@@ -3918,7 +3810,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
         <v>232</v>
       </c>
@@ -4933,7 +4825,7 @@
       <c r="A151" s="1" t="s">
         <v>357</v>
       </c>
-      <c r="B151" s="7" t="s">
+      <c r="B151" s="1" t="s">
         <v>332</v>
       </c>
       <c r="C151" s="1" t="s">
@@ -4983,7 +4875,7 @@
         <v>43</v>
       </c>
       <c r="E153" s="1" t="s">
-        <v>363</v>
+        <v>44</v>
       </c>
       <c r="F153" s="1" t="n">
         <v>0</v>
@@ -4991,19 +4883,19 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B154" s="7" t="s">
         <v>332</v>
       </c>
       <c r="C154" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="D154" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E154" s="1" t="s">
         <v>365</v>
-      </c>
-      <c r="D154" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E154" s="1" t="s">
-        <v>150</v>
       </c>
       <c r="F154" s="1" t="n">
         <v>0</v>
@@ -5023,7 +4915,7 @@
         <v>43</v>
       </c>
       <c r="E155" s="1" t="s">
-        <v>70</v>
+        <v>150</v>
       </c>
       <c r="F155" s="1" t="n">
         <v>0</v>
@@ -5036,7 +4928,7 @@
       <c r="B156" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="C156" s="7" t="s">
+      <c r="C156" s="1" t="s">
         <v>369</v>
       </c>
       <c r="D156" s="1" t="s">
@@ -5076,14 +4968,14 @@
       <c r="B158" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="C158" s="1" t="s">
+      <c r="C158" s="7" t="s">
         <v>373</v>
       </c>
       <c r="D158" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E158" s="1" t="s">
-        <v>363</v>
+        <v>70</v>
       </c>
       <c r="F158" s="1" t="n">
         <v>0</v>
@@ -5103,13 +4995,32 @@
         <v>43</v>
       </c>
       <c r="E159" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="F159" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A160" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="B160" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="D160" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E160" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F159" s="1" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+      <c r="F160" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>